<commit_message>
feat: add Hydraulic Structures asset group and update risk data
- Add new "Hydraulic Structures" asset group containing embankments, mainCanals, branchCanals, drains
- Move hydraulic assets from Infrastructure group to new dedicated group
- Update asset grouping in DistrictBarChart, EadBarChart, and RiskEadView
- Update risk.json with latest Excel values

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/risk/Risk_Analysis_T3_2.3yrs_Future_Breaches.xlsx
+++ b/risk/Risk_Analysis_T3_2.3yrs_Future_Breaches.xlsx
@@ -560,7 +560,7 @@
         <v>30870</v>
       </c>
       <c r="H4" t="n">
-        <v>1470</v>
+        <v>2310</v>
       </c>
       <c r="I4" t="n">
         <v>1</v>
@@ -572,22 +572,22 @@
         <v>4</v>
       </c>
       <c r="L4" t="n">
-        <v>98610</v>
+        <v>97800</v>
       </c>
       <c r="M4" t="n">
-        <v>25920</v>
+        <v>34110</v>
       </c>
       <c r="N4" t="n">
-        <v>2610</v>
+        <v>4440</v>
       </c>
       <c r="O4" t="n">
-        <v>13590</v>
+        <v>13080</v>
       </c>
       <c r="P4" t="n">
-        <v>28080</v>
+        <v>19290</v>
       </c>
       <c r="Q4" t="n">
-        <v>12381.13</v>
+        <v>128304.42</v>
       </c>
     </row>
     <row r="5">
@@ -613,7 +613,7 @@
         <v>25770</v>
       </c>
       <c r="H5" t="n">
-        <v>1890</v>
+        <v>1770</v>
       </c>
       <c r="I5" t="n">
         <v>1</v>
@@ -625,22 +625,22 @@
         <v>11</v>
       </c>
       <c r="L5" t="n">
-        <v>93690</v>
+        <v>108390</v>
       </c>
       <c r="M5" t="n">
-        <v>14670</v>
+        <v>35430</v>
       </c>
       <c r="N5" t="n">
-        <v>1410</v>
+        <v>1530</v>
       </c>
       <c r="O5" t="n">
-        <v>10350</v>
+        <v>11910</v>
       </c>
       <c r="P5" t="n">
-        <v>43230</v>
+        <v>32670</v>
       </c>
       <c r="Q5" t="n">
-        <v>16742.46</v>
+        <v>173500.44</v>
       </c>
     </row>
     <row r="6">
@@ -666,7 +666,7 @@
         <v>20220</v>
       </c>
       <c r="H6" t="n">
-        <v>3360</v>
+        <v>3840</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
@@ -678,22 +678,22 @@
         <v>2</v>
       </c>
       <c r="L6" t="n">
-        <v>62640</v>
+        <v>84450</v>
       </c>
       <c r="M6" t="n">
-        <v>6240</v>
+        <v>21720</v>
       </c>
       <c r="N6" t="n">
-        <v>180</v>
+        <v>450</v>
       </c>
       <c r="O6" t="n">
-        <v>1620</v>
+        <v>3660</v>
       </c>
       <c r="P6" t="n">
-        <v>37680</v>
+        <v>39180</v>
       </c>
       <c r="Q6" t="n">
-        <v>18458.97</v>
+        <v>191288.57</v>
       </c>
     </row>
     <row r="7">
@@ -719,7 +719,7 @@
         <v>12300</v>
       </c>
       <c r="H7" t="n">
-        <v>90</v>
+        <v>450</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
@@ -731,22 +731,22 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>35520</v>
+        <v>61560</v>
       </c>
       <c r="M7" t="n">
-        <v>3210</v>
+        <v>17220</v>
       </c>
       <c r="N7" t="n">
         <v>0</v>
       </c>
       <c r="O7" t="n">
-        <v>180</v>
+        <v>390</v>
       </c>
       <c r="P7" t="n">
-        <v>33690</v>
+        <v>44940</v>
       </c>
       <c r="Q7" t="n">
-        <v>13738.96</v>
+        <v>142375.56</v>
       </c>
     </row>
     <row r="8">
@@ -784,10 +784,10 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>17220</v>
+        <v>36690</v>
       </c>
       <c r="M8" t="n">
-        <v>3210</v>
+        <v>9510</v>
       </c>
       <c r="N8" t="n">
         <v>0</v>
@@ -796,10 +796,10 @@
         <v>0</v>
       </c>
       <c r="P8" t="n">
-        <v>22320</v>
+        <v>33420</v>
       </c>
       <c r="Q8" t="n">
-        <v>8480.93</v>
+        <v>87887.06</v>
       </c>
     </row>
     <row r="9">
@@ -825,7 +825,7 @@
         <v>2370</v>
       </c>
       <c r="H9" t="n">
-        <v>60</v>
+        <v>180</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
@@ -837,22 +837,22 @@
         <v>2</v>
       </c>
       <c r="L9" t="n">
-        <v>5040</v>
+        <v>21780</v>
       </c>
       <c r="M9" t="n">
-        <v>960</v>
+        <v>4110</v>
       </c>
       <c r="N9" t="n">
         <v>0</v>
       </c>
       <c r="O9" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="P9" t="n">
-        <v>23310</v>
+        <v>40080</v>
       </c>
       <c r="Q9" t="n">
-        <v>4515.89</v>
+        <v>46797.77</v>
       </c>
     </row>
     <row r="10">
@@ -890,10 +890,10 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>2130</v>
+        <v>7170</v>
       </c>
       <c r="M10" t="n">
-        <v>210</v>
+        <v>2490</v>
       </c>
       <c r="N10" t="n">
         <v>0</v>
@@ -902,10 +902,10 @@
         <v>0</v>
       </c>
       <c r="P10" t="n">
-        <v>7980</v>
+        <v>15450</v>
       </c>
       <c r="Q10" t="n">
-        <v>2254.99</v>
+        <v>23368.24</v>
       </c>
     </row>
     <row r="11">
@@ -943,10 +943,10 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>1470</v>
+        <v>3750</v>
       </c>
       <c r="M11" t="n">
-        <v>0</v>
+        <v>5040</v>
       </c>
       <c r="N11" t="n">
         <v>0</v>
@@ -955,10 +955,10 @@
         <v>0</v>
       </c>
       <c r="P11" t="n">
-        <v>5160</v>
+        <v>13920</v>
       </c>
       <c r="Q11" t="n">
-        <v>1353.37</v>
+        <v>14024.88</v>
       </c>
     </row>
     <row r="12">
@@ -996,10 +996,10 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>360</v>
+        <v>2040</v>
       </c>
       <c r="M12" t="n">
-        <v>0</v>
+        <v>930</v>
       </c>
       <c r="N12" t="n">
         <v>0</v>
@@ -1008,10 +1008,10 @@
         <v>0</v>
       </c>
       <c r="P12" t="n">
-        <v>660</v>
+        <v>2100</v>
       </c>
       <c r="Q12" t="n">
-        <v>1033.75</v>
+        <v>10712.66</v>
       </c>
     </row>
     <row r="13">
@@ -1037,7 +1037,7 @@
         <v>150</v>
       </c>
       <c r="H13" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="I13" t="n">
         <v>0</v>
@@ -1049,10 +1049,10 @@
         <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>240</v>
+        <v>660</v>
       </c>
       <c r="M13" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="N13" t="n">
         <v>0</v>
@@ -1061,10 +1061,10 @@
         <v>0</v>
       </c>
       <c r="P13" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="Q13" t="n">
-        <v>1044.24</v>
+        <v>10821.37</v>
       </c>
     </row>
     <row r="14">
@@ -1102,10 +1102,10 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>540</v>
+        <v>1410</v>
       </c>
       <c r="M14" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="N14" t="n">
         <v>0</v>
@@ -1117,7 +1117,7 @@
         <v>0</v>
       </c>
       <c r="Q14" t="n">
-        <v>1088.21</v>
+        <v>11277.03</v>
       </c>
     </row>
     <row r="15">
@@ -1155,10 +1155,10 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>0</v>
+        <v>960</v>
       </c>
       <c r="M15" t="n">
-        <v>0</v>
+        <v>240</v>
       </c>
       <c r="N15" t="n">
         <v>0</v>
@@ -1170,7 +1170,7 @@
         <v>0</v>
       </c>
       <c r="Q15" t="n">
-        <v>465.48</v>
+        <v>4823.76</v>
       </c>
     </row>
     <row r="16">
@@ -1208,7 +1208,7 @@
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>0</v>
+        <v>360</v>
       </c>
       <c r="M16" t="n">
         <v>0</v>
@@ -1223,7 +1223,7 @@
         <v>0</v>
       </c>
       <c r="Q16" t="n">
-        <v>174.21</v>
+        <v>1805.3</v>
       </c>
     </row>
     <row r="17">
@@ -1261,7 +1261,7 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="M17" t="n">
         <v>0</v>
@@ -1276,7 +1276,7 @@
         <v>0</v>
       </c>
       <c r="Q17" t="n">
-        <v>36.83</v>
+        <v>381.64</v>
       </c>
     </row>
     <row r="18">
@@ -1314,7 +1314,7 @@
         <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="M18" t="n">
         <v>0</v>
@@ -1329,7 +1329,7 @@
         <v>0</v>
       </c>
       <c r="Q18" t="n">
-        <v>3.68</v>
+        <v>38.16</v>
       </c>
     </row>
     <row r="19">
@@ -1382,7 +1382,7 @@
         <v>0</v>
       </c>
       <c r="Q19" t="n">
-        <v>0.22</v>
+        <v>2.31</v>
       </c>
     </row>
     <row r="20">
@@ -1852,7 +1852,7 @@
         <v>15630</v>
       </c>
       <c r="H4" t="n">
-        <v>1260</v>
+        <v>2010</v>
       </c>
       <c r="I4" t="n">
         <v>0</v>
@@ -1864,13 +1864,13 @@
         <v>2</v>
       </c>
       <c r="L4" t="n">
-        <v>32010</v>
+        <v>40080</v>
       </c>
       <c r="M4" t="n">
-        <v>6660</v>
+        <v>8520</v>
       </c>
       <c r="N4" t="n">
-        <v>30</v>
+        <v>570</v>
       </c>
       <c r="O4" t="n">
         <v>0</v>
@@ -1879,7 +1879,7 @@
         <v>0</v>
       </c>
       <c r="Q4" t="n">
-        <v>873.77</v>
+        <v>99027.72</v>
       </c>
     </row>
     <row r="5">
@@ -1905,7 +1905,7 @@
         <v>12450</v>
       </c>
       <c r="H5" t="n">
-        <v>1890</v>
+        <v>1650</v>
       </c>
       <c r="I5" t="n">
         <v>1</v>
@@ -1917,13 +1917,13 @@
         <v>7</v>
       </c>
       <c r="L5" t="n">
-        <v>30480</v>
+        <v>35160</v>
       </c>
       <c r="M5" t="n">
-        <v>8010</v>
+        <v>12210</v>
       </c>
       <c r="N5" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="O5" t="n">
         <v>0</v>
@@ -1932,7 +1932,7 @@
         <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>1043.66</v>
+        <v>118281.24</v>
       </c>
     </row>
     <row r="6">
@@ -1958,7 +1958,7 @@
         <v>6750</v>
       </c>
       <c r="H6" t="n">
-        <v>3360</v>
+        <v>3840</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
@@ -1970,10 +1970,10 @@
         <v>1</v>
       </c>
       <c r="L6" t="n">
-        <v>22110</v>
+        <v>28230</v>
       </c>
       <c r="M6" t="n">
-        <v>3660</v>
+        <v>7050</v>
       </c>
       <c r="N6" t="n">
         <v>0</v>
@@ -1985,7 +1985,7 @@
         <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>1210.19</v>
+        <v>137155.32</v>
       </c>
     </row>
     <row r="7">
@@ -2011,7 +2011,7 @@
         <v>3570</v>
       </c>
       <c r="H7" t="n">
-        <v>90</v>
+        <v>450</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
@@ -2023,10 +2023,10 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>9270</v>
+        <v>14910</v>
       </c>
       <c r="M7" t="n">
-        <v>2460</v>
+        <v>4140</v>
       </c>
       <c r="N7" t="n">
         <v>0</v>
@@ -2038,7 +2038,7 @@
         <v>0</v>
       </c>
       <c r="Q7" t="n">
-        <v>1067.23</v>
+        <v>120952.62</v>
       </c>
     </row>
     <row r="8">
@@ -2076,10 +2076,10 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>5250</v>
+        <v>9360</v>
       </c>
       <c r="M8" t="n">
-        <v>2940</v>
+        <v>4620</v>
       </c>
       <c r="N8" t="n">
         <v>0</v>
@@ -2091,7 +2091,7 @@
         <v>0</v>
       </c>
       <c r="Q8" t="n">
-        <v>677.51</v>
+        <v>76784.58</v>
       </c>
     </row>
     <row r="9">
@@ -2117,7 +2117,7 @@
         <v>870</v>
       </c>
       <c r="H9" t="n">
-        <v>60</v>
+        <v>180</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
@@ -2129,10 +2129,10 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>1500</v>
+        <v>2490</v>
       </c>
       <c r="M9" t="n">
-        <v>600</v>
+        <v>1200</v>
       </c>
       <c r="N9" t="n">
         <v>0</v>
@@ -2144,7 +2144,7 @@
         <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>305.59</v>
+        <v>34633.08</v>
       </c>
     </row>
     <row r="10">
@@ -2182,10 +2182,10 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>660</v>
+        <v>1170</v>
       </c>
       <c r="M10" t="n">
-        <v>60</v>
+        <v>840</v>
       </c>
       <c r="N10" t="n">
         <v>0</v>
@@ -2197,7 +2197,7 @@
         <v>0</v>
       </c>
       <c r="Q10" t="n">
-        <v>132.44</v>
+        <v>15009.3</v>
       </c>
     </row>
     <row r="11">
@@ -2235,10 +2235,10 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>1170</v>
+        <v>2370</v>
       </c>
       <c r="M11" t="n">
-        <v>0</v>
+        <v>1770</v>
       </c>
       <c r="N11" t="n">
         <v>0</v>
@@ -2250,7 +2250,7 @@
         <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>88.20999999999999</v>
+        <v>9997.02</v>
       </c>
     </row>
     <row r="12">
@@ -2288,10 +2288,10 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>240</v>
+        <v>1290</v>
       </c>
       <c r="M12" t="n">
-        <v>0</v>
+        <v>660</v>
       </c>
       <c r="N12" t="n">
         <v>0</v>
@@ -2303,7 +2303,7 @@
         <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>72.95</v>
+        <v>8268.120000000001</v>
       </c>
     </row>
     <row r="13">
@@ -2329,7 +2329,7 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="I13" t="n">
         <v>0</v>
@@ -2341,11 +2341,11 @@
         <v>0</v>
       </c>
       <c r="L13" t="n">
+        <v>420</v>
+      </c>
+      <c r="M13" t="n">
         <v>90</v>
       </c>
-      <c r="M13" t="n">
-        <v>0</v>
-      </c>
       <c r="N13" t="n">
         <v>0</v>
       </c>
@@ -2356,7 +2356,7 @@
         <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>85.54000000000001</v>
+        <v>9694.08</v>
       </c>
     </row>
     <row r="14">
@@ -2394,10 +2394,10 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>0</v>
+        <v>780</v>
       </c>
       <c r="M14" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="N14" t="n">
         <v>0</v>
@@ -2409,7 +2409,7 @@
         <v>0</v>
       </c>
       <c r="Q14" t="n">
-        <v>95.93000000000001</v>
+        <v>10872.18</v>
       </c>
     </row>
     <row r="15">
@@ -2447,10 +2447,10 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>0</v>
+        <v>960</v>
       </c>
       <c r="M15" t="n">
-        <v>0</v>
+        <v>240</v>
       </c>
       <c r="N15" t="n">
         <v>0</v>
@@ -2462,7 +2462,7 @@
         <v>0</v>
       </c>
       <c r="Q15" t="n">
-        <v>38.04</v>
+        <v>4311.54</v>
       </c>
     </row>
     <row r="16">
@@ -2500,7 +2500,7 @@
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>0</v>
+        <v>360</v>
       </c>
       <c r="M16" t="n">
         <v>0</v>
@@ -2515,7 +2515,7 @@
         <v>0</v>
       </c>
       <c r="Q16" t="n">
-        <v>29</v>
+        <v>3286.44</v>
       </c>
     </row>
     <row r="17">
@@ -2553,7 +2553,7 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="M17" t="n">
         <v>0</v>
@@ -2568,7 +2568,7 @@
         <v>0</v>
       </c>
       <c r="Q17" t="n">
-        <v>0.43</v>
+        <v>48.96</v>
       </c>
     </row>
     <row r="18">
@@ -2606,7 +2606,7 @@
         <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="M18" t="n">
         <v>0</v>
@@ -2621,7 +2621,7 @@
         <v>0</v>
       </c>
       <c r="Q18" t="n">
-        <v>0.51</v>
+        <v>58.14</v>
       </c>
     </row>
     <row r="19">
@@ -3197,7 +3197,7 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>680.4</v>
+        <v>594</v>
       </c>
       <c r="I5" t="n">
         <v>0.33</v>
@@ -3209,13 +3209,13 @@
         <v>2.32</v>
       </c>
       <c r="L5" t="n">
-        <v>6400.8</v>
+        <v>7383.6</v>
       </c>
       <c r="M5" t="n">
-        <v>160.2</v>
+        <v>244.2</v>
       </c>
       <c r="N5" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="O5" t="n">
         <v>0</v>
@@ -3224,7 +3224,7 @@
         <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>52.18</v>
+        <v>5914.06</v>
       </c>
     </row>
     <row r="6">
@@ -3250,7 +3250,7 @@
         <v>337.5</v>
       </c>
       <c r="H6" t="n">
-        <v>1915.2</v>
+        <v>2188.8</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
@@ -3262,10 +3262,10 @@
         <v>0.51</v>
       </c>
       <c r="L6" t="n">
-        <v>8180.7</v>
+        <v>10445.1</v>
       </c>
       <c r="M6" t="n">
-        <v>292.8</v>
+        <v>564</v>
       </c>
       <c r="N6" t="n">
         <v>0</v>
@@ -3277,7 +3277,7 @@
         <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>907.65</v>
+        <v>102866.49</v>
       </c>
     </row>
     <row r="7">
@@ -3303,7 +3303,7 @@
         <v>535.5</v>
       </c>
       <c r="H7" t="n">
-        <v>65.7</v>
+        <v>328.5</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
@@ -3315,10 +3315,10 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>5562</v>
+        <v>8946</v>
       </c>
       <c r="M7" t="n">
-        <v>861</v>
+        <v>1449</v>
       </c>
       <c r="N7" t="n">
         <v>0</v>
@@ -3330,7 +3330,7 @@
         <v>0</v>
       </c>
       <c r="Q7" t="n">
-        <v>853.78</v>
+        <v>96762.10000000001</v>
       </c>
     </row>
     <row r="8">
@@ -3368,10 +3368,10 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>3727.5</v>
+        <v>6645.6</v>
       </c>
       <c r="M8" t="n">
-        <v>1617</v>
+        <v>2541</v>
       </c>
       <c r="N8" t="n">
         <v>0</v>
@@ -3383,7 +3383,7 @@
         <v>0</v>
       </c>
       <c r="Q8" t="n">
-        <v>643.64</v>
+        <v>72945.35000000001</v>
       </c>
     </row>
     <row r="9">
@@ -3409,7 +3409,7 @@
         <v>739.5</v>
       </c>
       <c r="H9" t="n">
-        <v>60</v>
+        <v>180</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
@@ -3421,10 +3421,10 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>1215</v>
+        <v>2016.9</v>
       </c>
       <c r="M9" t="n">
-        <v>420</v>
+        <v>840</v>
       </c>
       <c r="N9" t="n">
         <v>0</v>
@@ -3436,7 +3436,7 @@
         <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>296.42</v>
+        <v>33594.09</v>
       </c>
     </row>
     <row r="10">
@@ -3474,10 +3474,10 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>587.4</v>
+        <v>1041.3</v>
       </c>
       <c r="M10" t="n">
-        <v>51</v>
+        <v>714</v>
       </c>
       <c r="N10" t="n">
         <v>0</v>
@@ -3489,7 +3489,7 @@
         <v>0</v>
       </c>
       <c r="Q10" t="n">
-        <v>132.44</v>
+        <v>15009.3</v>
       </c>
     </row>
     <row r="11">
@@ -3527,10 +3527,10 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>1170</v>
+        <v>2370</v>
       </c>
       <c r="M11" t="n">
-        <v>0</v>
+        <v>1593</v>
       </c>
       <c r="N11" t="n">
         <v>0</v>
@@ -3542,7 +3542,7 @@
         <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>88.20999999999999</v>
+        <v>9997.02</v>
       </c>
     </row>
     <row r="12">
@@ -3580,10 +3580,10 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>240</v>
+        <v>1290</v>
       </c>
       <c r="M12" t="n">
-        <v>0</v>
+        <v>627</v>
       </c>
       <c r="N12" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
         <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>72.95</v>
+        <v>8268.120000000001</v>
       </c>
     </row>
     <row r="13">
@@ -3621,7 +3621,7 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="I13" t="n">
         <v>0</v>
@@ -3633,11 +3633,11 @@
         <v>0</v>
       </c>
       <c r="L13" t="n">
+        <v>420</v>
+      </c>
+      <c r="M13" t="n">
         <v>90</v>
       </c>
-      <c r="M13" t="n">
-        <v>0</v>
-      </c>
       <c r="N13" t="n">
         <v>0</v>
       </c>
@@ -3648,7 +3648,7 @@
         <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>85.54000000000001</v>
+        <v>9694.08</v>
       </c>
     </row>
     <row r="14">
@@ -3686,10 +3686,10 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>0</v>
+        <v>780</v>
       </c>
       <c r="M14" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="N14" t="n">
         <v>0</v>
@@ -3701,7 +3701,7 @@
         <v>0</v>
       </c>
       <c r="Q14" t="n">
-        <v>95.93000000000001</v>
+        <v>10872.18</v>
       </c>
     </row>
     <row r="15">
@@ -3739,10 +3739,10 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>0</v>
+        <v>960</v>
       </c>
       <c r="M15" t="n">
-        <v>0</v>
+        <v>240</v>
       </c>
       <c r="N15" t="n">
         <v>0</v>
@@ -3754,7 +3754,7 @@
         <v>0</v>
       </c>
       <c r="Q15" t="n">
-        <v>38.04</v>
+        <v>4311.54</v>
       </c>
     </row>
     <row r="16">
@@ -3792,7 +3792,7 @@
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>0</v>
+        <v>360</v>
       </c>
       <c r="M16" t="n">
         <v>0</v>
@@ -3807,7 +3807,7 @@
         <v>0</v>
       </c>
       <c r="Q16" t="n">
-        <v>29</v>
+        <v>3286.44</v>
       </c>
     </row>
     <row r="17">
@@ -3845,7 +3845,7 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="M17" t="n">
         <v>0</v>
@@ -3860,7 +3860,7 @@
         <v>0</v>
       </c>
       <c r="Q17" t="n">
-        <v>0.43</v>
+        <v>48.96</v>
       </c>
     </row>
     <row r="18">
@@ -3898,7 +3898,7 @@
         <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="M18" t="n">
         <v>0</v>
@@ -3913,7 +3913,7 @@
         <v>0</v>
       </c>
       <c r="Q18" t="n">
-        <v>0.51</v>
+        <v>58.14</v>
       </c>
     </row>
     <row r="19">
@@ -4489,7 +4489,7 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>3878280</v>
+        <v>3385800</v>
       </c>
       <c r="I5" t="n">
         <v>64288.14</v>
@@ -4501,13 +4501,13 @@
         <v>112504.25</v>
       </c>
       <c r="L5" t="n">
-        <v>1152144</v>
+        <v>1329048</v>
       </c>
       <c r="M5" t="n">
-        <v>56070</v>
+        <v>85470</v>
       </c>
       <c r="N5" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="O5" t="n">
         <v>0</v>
@@ -4516,7 +4516,7 @@
         <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>31309.74</v>
+        <v>3548437.2</v>
       </c>
     </row>
     <row r="6">
@@ -4542,7 +4542,7 @@
         <v>18225</v>
       </c>
       <c r="H6" t="n">
-        <v>10916640</v>
+        <v>12476160</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
@@ -4554,10 +4554,10 @@
         <v>24617.89</v>
       </c>
       <c r="L6" t="n">
-        <v>1472526</v>
+        <v>1880118</v>
       </c>
       <c r="M6" t="n">
-        <v>102480</v>
+        <v>197400</v>
       </c>
       <c r="N6" t="n">
         <v>0</v>
@@ -4569,7 +4569,7 @@
         <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>544587.3</v>
+        <v>61719894</v>
       </c>
     </row>
     <row r="7">
@@ -4595,7 +4595,7 @@
         <v>28917</v>
       </c>
       <c r="H7" t="n">
-        <v>374490</v>
+        <v>1872450</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
@@ -4607,10 +4607,10 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>1001160</v>
+        <v>1610280</v>
       </c>
       <c r="M7" t="n">
-        <v>301350</v>
+        <v>507150</v>
       </c>
       <c r="N7" t="n">
         <v>0</v>
@@ -4622,7 +4622,7 @@
         <v>0</v>
       </c>
       <c r="Q7" t="n">
-        <v>512269.92</v>
+        <v>58057257.6</v>
       </c>
     </row>
     <row r="8">
@@ -4660,10 +4660,10 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>670950</v>
+        <v>1196208</v>
       </c>
       <c r="M8" t="n">
-        <v>565950</v>
+        <v>889350</v>
       </c>
       <c r="N8" t="n">
         <v>0</v>
@@ -4675,7 +4675,7 @@
         <v>0</v>
       </c>
       <c r="Q8" t="n">
-        <v>386181.27</v>
+        <v>43767210.6</v>
       </c>
     </row>
     <row r="9">
@@ -4701,7 +4701,7 @@
         <v>39933</v>
       </c>
       <c r="H9" t="n">
-        <v>342000</v>
+        <v>1026000</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
@@ -4713,10 +4713,10 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>218700</v>
+        <v>363042</v>
       </c>
       <c r="M9" t="n">
-        <v>147000</v>
+        <v>294000</v>
       </c>
       <c r="N9" t="n">
         <v>0</v>
@@ -4728,7 +4728,7 @@
         <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>177851.05</v>
+        <v>20156452.56</v>
       </c>
     </row>
     <row r="10">
@@ -4766,10 +4766,10 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>105732</v>
+        <v>187434</v>
       </c>
       <c r="M10" t="n">
-        <v>17850</v>
+        <v>249900</v>
       </c>
       <c r="N10" t="n">
         <v>0</v>
@@ -4781,7 +4781,7 @@
         <v>0</v>
       </c>
       <c r="Q10" t="n">
-        <v>79461</v>
+        <v>9005580</v>
       </c>
     </row>
     <row r="11">
@@ -4819,10 +4819,10 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>210600</v>
+        <v>426600</v>
       </c>
       <c r="M11" t="n">
-        <v>0</v>
+        <v>557550</v>
       </c>
       <c r="N11" t="n">
         <v>0</v>
@@ -4834,7 +4834,7 @@
         <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>52925.4</v>
+        <v>5998212</v>
       </c>
     </row>
     <row r="12">
@@ -4872,10 +4872,10 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>43200</v>
+        <v>232200</v>
       </c>
       <c r="M12" t="n">
-        <v>0</v>
+        <v>219450</v>
       </c>
       <c r="N12" t="n">
         <v>0</v>
@@ -4887,7 +4887,7 @@
         <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>43772.4</v>
+        <v>4960872</v>
       </c>
     </row>
     <row r="13">
@@ -4913,7 +4913,7 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>171000</v>
+        <v>513000</v>
       </c>
       <c r="I13" t="n">
         <v>0</v>
@@ -4925,10 +4925,10 @@
         <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>16200</v>
+        <v>75600</v>
       </c>
       <c r="M13" t="n">
-        <v>0</v>
+        <v>31500</v>
       </c>
       <c r="N13" t="n">
         <v>0</v>
@@ -4940,7 +4940,7 @@
         <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>51321.6</v>
+        <v>5816448</v>
       </c>
     </row>
     <row r="14">
@@ -4978,10 +4978,10 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>0</v>
+        <v>140400</v>
       </c>
       <c r="M14" t="n">
-        <v>0</v>
+        <v>52500</v>
       </c>
       <c r="N14" t="n">
         <v>0</v>
@@ -4993,7 +4993,7 @@
         <v>0</v>
       </c>
       <c r="Q14" t="n">
-        <v>57558.6</v>
+        <v>6523308</v>
       </c>
     </row>
     <row r="15">
@@ -5031,10 +5031,10 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>0</v>
+        <v>172800</v>
       </c>
       <c r="M15" t="n">
-        <v>0</v>
+        <v>84000</v>
       </c>
       <c r="N15" t="n">
         <v>0</v>
@@ -5046,7 +5046,7 @@
         <v>0</v>
       </c>
       <c r="Q15" t="n">
-        <v>22825.8</v>
+        <v>2586924</v>
       </c>
     </row>
     <row r="16">
@@ -5084,7 +5084,7 @@
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>0</v>
+        <v>64800</v>
       </c>
       <c r="M16" t="n">
         <v>0</v>
@@ -5099,7 +5099,7 @@
         <v>0</v>
       </c>
       <c r="Q16" t="n">
-        <v>17398.8</v>
+        <v>1971864</v>
       </c>
     </row>
     <row r="17">
@@ -5137,7 +5137,7 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>0</v>
+        <v>16200</v>
       </c>
       <c r="M17" t="n">
         <v>0</v>
@@ -5152,7 +5152,7 @@
         <v>0</v>
       </c>
       <c r="Q17" t="n">
-        <v>259.2</v>
+        <v>29376</v>
       </c>
     </row>
     <row r="18">
@@ -5190,7 +5190,7 @@
         <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>0</v>
+        <v>27000</v>
       </c>
       <c r="M18" t="n">
         <v>0</v>
@@ -5205,7 +5205,7 @@
         <v>0</v>
       </c>
       <c r="Q18" t="n">
-        <v>307.8</v>
+        <v>34884</v>
       </c>
     </row>
     <row r="19">
@@ -5752,10 +5752,10 @@
         <v>0</v>
       </c>
       <c r="P4" t="n">
-        <v>90</v>
+        <v>330</v>
       </c>
       <c r="Q4" t="n">
-        <v>2.46</v>
+        <v>12.96</v>
       </c>
     </row>
     <row r="5">
@@ -9625,13 +9625,13 @@
         <v>0</v>
       </c>
       <c r="O4" t="n">
-        <v>270</v>
+        <v>570</v>
       </c>
       <c r="P4" t="n">
         <v>0</v>
       </c>
       <c r="Q4" t="n">
-        <v>79.41</v>
+        <v>430.92</v>
       </c>
     </row>
     <row r="5">
@@ -13492,19 +13492,19 @@
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>32550</v>
+        <v>21930</v>
       </c>
       <c r="M4" t="n">
-        <v>6090</v>
+        <v>5310</v>
       </c>
       <c r="N4" t="n">
         <v>0</v>
       </c>
       <c r="O4" t="n">
-        <v>9120</v>
+        <v>8010</v>
       </c>
       <c r="P4" t="n">
-        <v>8100</v>
+        <v>11610</v>
       </c>
       <c r="Q4" t="n">
         <v>2627.96</v>
@@ -13545,19 +13545,19 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>18900</v>
+        <v>24990</v>
       </c>
       <c r="M5" t="n">
-        <v>2850</v>
+        <v>12570</v>
       </c>
       <c r="N5" t="n">
         <v>0</v>
       </c>
       <c r="O5" t="n">
-        <v>9660</v>
+        <v>10680</v>
       </c>
       <c r="P5" t="n">
-        <v>13500</v>
+        <v>5400</v>
       </c>
       <c r="Q5" t="n">
         <v>516.8200000000001</v>
@@ -13598,19 +13598,19 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>6690</v>
+        <v>17790</v>
       </c>
       <c r="M6" t="n">
-        <v>1080</v>
+        <v>9420</v>
       </c>
       <c r="N6" t="n">
         <v>0</v>
       </c>
       <c r="O6" t="n">
-        <v>1560</v>
+        <v>3540</v>
       </c>
       <c r="P6" t="n">
-        <v>16650</v>
+        <v>10260</v>
       </c>
       <c r="Q6" t="n">
         <v>93.97</v>
@@ -13651,19 +13651,19 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>2610</v>
+        <v>17760</v>
       </c>
       <c r="M7" t="n">
+        <v>7440</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" t="n">
         <v>300</v>
       </c>
-      <c r="N7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O7" t="n">
-        <v>180</v>
-      </c>
       <c r="P7" t="n">
-        <v>14970</v>
+        <v>18180</v>
       </c>
       <c r="Q7" t="n">
         <v>32.36</v>
@@ -13704,10 +13704,10 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>2010</v>
+        <v>14340</v>
       </c>
       <c r="M8" t="n">
-        <v>150</v>
+        <v>3420</v>
       </c>
       <c r="N8" t="n">
         <v>0</v>
@@ -13716,7 +13716,7 @@
         <v>0</v>
       </c>
       <c r="P8" t="n">
-        <v>14820</v>
+        <v>20040</v>
       </c>
       <c r="Q8" t="n">
         <v>29.46</v>
@@ -13757,19 +13757,19 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>1530</v>
+        <v>15900</v>
       </c>
       <c r="M9" t="n">
-        <v>150</v>
+        <v>1440</v>
       </c>
       <c r="N9" t="n">
         <v>0</v>
       </c>
       <c r="O9" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="P9" t="n">
-        <v>16560</v>
+        <v>28770</v>
       </c>
       <c r="Q9" t="n">
         <v>20.53</v>
@@ -13810,10 +13810,10 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>540</v>
+        <v>4680</v>
       </c>
       <c r="M10" t="n">
-        <v>120</v>
+        <v>180</v>
       </c>
       <c r="N10" t="n">
         <v>0</v>
@@ -13822,7 +13822,7 @@
         <v>0</v>
       </c>
       <c r="P10" t="n">
-        <v>5190</v>
+        <v>12270</v>
       </c>
       <c r="Q10" t="n">
         <v>6.25</v>
@@ -13863,7 +13863,7 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>0</v>
+        <v>1050</v>
       </c>
       <c r="M11" t="n">
         <v>0</v>
@@ -13875,7 +13875,7 @@
         <v>0</v>
       </c>
       <c r="P11" t="n">
-        <v>1410</v>
+        <v>5100</v>
       </c>
       <c r="Q11" t="n">
         <v>2.79</v>
@@ -13916,7 +13916,7 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>30</v>
+        <v>390</v>
       </c>
       <c r="M12" t="n">
         <v>0</v>
@@ -13928,7 +13928,7 @@
         <v>0</v>
       </c>
       <c r="P12" t="n">
-        <v>120</v>
+        <v>570</v>
       </c>
       <c r="Q12" t="n">
         <v>1</v>
@@ -13969,7 +13969,7 @@
         <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="M13" t="n">
         <v>0</v>
@@ -13981,7 +13981,7 @@
         <v>0</v>
       </c>
       <c r="P13" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="Q13" t="n">
         <v>0.11</v>
@@ -14825,7 +14825,7 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>680.4</v>
+        <v>637.2</v>
       </c>
       <c r="I5" t="n">
         <v>0.33</v>
@@ -14837,22 +14837,22 @@
         <v>3.64</v>
       </c>
       <c r="L5" t="n">
-        <v>19674.9</v>
+        <v>22761.9</v>
       </c>
       <c r="M5" t="n">
-        <v>293.4</v>
+        <v>708.6</v>
       </c>
       <c r="N5" t="n">
-        <v>14.1</v>
+        <v>15.3</v>
       </c>
       <c r="O5" t="n">
-        <v>517.5</v>
+        <v>595.5</v>
       </c>
       <c r="P5" t="n">
-        <v>864.6</v>
+        <v>653.4</v>
       </c>
       <c r="Q5" t="n">
-        <v>837.12</v>
+        <v>8675.02</v>
       </c>
     </row>
     <row r="6">
@@ -14878,7 +14878,7 @@
         <v>1011</v>
       </c>
       <c r="H6" t="n">
-        <v>1915.2</v>
+        <v>2188.8</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
@@ -14890,22 +14890,22 @@
         <v>1.01</v>
       </c>
       <c r="L6" t="n">
-        <v>23176.8</v>
+        <v>31246.5</v>
       </c>
       <c r="M6" t="n">
-        <v>499.2</v>
+        <v>1737.6</v>
       </c>
       <c r="N6" t="n">
-        <v>9</v>
+        <v>22.5</v>
       </c>
       <c r="O6" t="n">
-        <v>405</v>
+        <v>915</v>
       </c>
       <c r="P6" t="n">
-        <v>5652</v>
+        <v>5877</v>
       </c>
       <c r="Q6" t="n">
-        <v>13844.23</v>
+        <v>143466.43</v>
       </c>
     </row>
     <row r="7">
@@ -14931,7 +14931,7 @@
         <v>1845</v>
       </c>
       <c r="H7" t="n">
-        <v>65.7</v>
+        <v>328.5</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
@@ -14943,22 +14943,22 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>21312</v>
+        <v>36936</v>
       </c>
       <c r="M7" t="n">
-        <v>1123.5</v>
+        <v>6027</v>
       </c>
       <c r="N7" t="n">
         <v>0</v>
       </c>
       <c r="O7" t="n">
-        <v>63</v>
+        <v>136.5</v>
       </c>
       <c r="P7" t="n">
-        <v>8422.5</v>
+        <v>11235</v>
       </c>
       <c r="Q7" t="n">
-        <v>10991.17</v>
+        <v>113900.45</v>
       </c>
     </row>
     <row r="8">
@@ -14996,10 +14996,10 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>12226.2</v>
+        <v>26049.9</v>
       </c>
       <c r="M8" t="n">
-        <v>1765.5</v>
+        <v>5230.5</v>
       </c>
       <c r="N8" t="n">
         <v>0</v>
@@ -15008,10 +15008,10 @@
         <v>0</v>
       </c>
       <c r="P8" t="n">
-        <v>8481.6</v>
+        <v>12699.6</v>
       </c>
       <c r="Q8" t="n">
-        <v>8056.88</v>
+        <v>83492.71000000001</v>
       </c>
     </row>
     <row r="9">
@@ -15037,7 +15037,7 @@
         <v>2014.5</v>
       </c>
       <c r="H9" t="n">
-        <v>60</v>
+        <v>180</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
@@ -15049,22 +15049,22 @@
         <v>1.61</v>
       </c>
       <c r="L9" t="n">
-        <v>4082.4</v>
+        <v>17641.8</v>
       </c>
       <c r="M9" t="n">
-        <v>672</v>
+        <v>2877</v>
       </c>
       <c r="N9" t="n">
         <v>0</v>
       </c>
       <c r="O9" t="n">
-        <v>0</v>
+        <v>16.5</v>
       </c>
       <c r="P9" t="n">
-        <v>11655</v>
+        <v>20040</v>
       </c>
       <c r="Q9" t="n">
-        <v>4380.42</v>
+        <v>45393.84</v>
       </c>
     </row>
     <row r="10">
@@ -15102,10 +15102,10 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>1895.7</v>
+        <v>6381.3</v>
       </c>
       <c r="M10" t="n">
-        <v>178.5</v>
+        <v>2116.5</v>
       </c>
       <c r="N10" t="n">
         <v>0</v>
@@ -15114,10 +15114,10 @@
         <v>0</v>
       </c>
       <c r="P10" t="n">
-        <v>6783</v>
+        <v>13132.5</v>
       </c>
       <c r="Q10" t="n">
-        <v>2254.99</v>
+        <v>23368.24</v>
       </c>
     </row>
     <row r="11">
@@ -15155,10 +15155,10 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>1470</v>
+        <v>3750</v>
       </c>
       <c r="M11" t="n">
-        <v>0</v>
+        <v>4536</v>
       </c>
       <c r="N11" t="n">
         <v>0</v>
@@ -15167,10 +15167,10 @@
         <v>0</v>
       </c>
       <c r="P11" t="n">
-        <v>4644</v>
+        <v>12528</v>
       </c>
       <c r="Q11" t="n">
-        <v>1353.37</v>
+        <v>14024.88</v>
       </c>
     </row>
     <row r="12">
@@ -15208,10 +15208,10 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>360</v>
+        <v>2040</v>
       </c>
       <c r="M12" t="n">
-        <v>0</v>
+        <v>883.5</v>
       </c>
       <c r="N12" t="n">
         <v>0</v>
@@ -15220,10 +15220,10 @@
         <v>0</v>
       </c>
       <c r="P12" t="n">
-        <v>660</v>
+        <v>2100</v>
       </c>
       <c r="Q12" t="n">
-        <v>1033.75</v>
+        <v>10712.66</v>
       </c>
     </row>
     <row r="13">
@@ -15249,7 +15249,7 @@
         <v>150</v>
       </c>
       <c r="H13" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="I13" t="n">
         <v>0</v>
@@ -15261,10 +15261,10 @@
         <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>240</v>
+        <v>660</v>
       </c>
       <c r="M13" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="N13" t="n">
         <v>0</v>
@@ -15273,10 +15273,10 @@
         <v>0</v>
       </c>
       <c r="P13" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="Q13" t="n">
-        <v>1044.24</v>
+        <v>10821.37</v>
       </c>
     </row>
     <row r="14">
@@ -15314,10 +15314,10 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>540</v>
+        <v>1410</v>
       </c>
       <c r="M14" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="N14" t="n">
         <v>0</v>
@@ -15329,7 +15329,7 @@
         <v>0</v>
       </c>
       <c r="Q14" t="n">
-        <v>1088.21</v>
+        <v>11277.03</v>
       </c>
     </row>
     <row r="15">
@@ -15367,10 +15367,10 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>0</v>
+        <v>960</v>
       </c>
       <c r="M15" t="n">
-        <v>0</v>
+        <v>240</v>
       </c>
       <c r="N15" t="n">
         <v>0</v>
@@ -15382,7 +15382,7 @@
         <v>0</v>
       </c>
       <c r="Q15" t="n">
-        <v>465.48</v>
+        <v>4823.76</v>
       </c>
     </row>
     <row r="16">
@@ -15420,7 +15420,7 @@
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>0</v>
+        <v>360</v>
       </c>
       <c r="M16" t="n">
         <v>0</v>
@@ -15435,7 +15435,7 @@
         <v>0</v>
       </c>
       <c r="Q16" t="n">
-        <v>174.21</v>
+        <v>1805.3</v>
       </c>
     </row>
     <row r="17">
@@ -15473,7 +15473,7 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="M17" t="n">
         <v>0</v>
@@ -15488,7 +15488,7 @@
         <v>0</v>
       </c>
       <c r="Q17" t="n">
-        <v>36.83</v>
+        <v>381.64</v>
       </c>
     </row>
     <row r="18">
@@ -15526,7 +15526,7 @@
         <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="M18" t="n">
         <v>0</v>
@@ -15541,7 +15541,7 @@
         <v>0</v>
       </c>
       <c r="Q18" t="n">
-        <v>3.68</v>
+        <v>38.16</v>
       </c>
     </row>
     <row r="19">
@@ -15594,7 +15594,7 @@
         <v>0</v>
       </c>
       <c r="Q19" t="n">
-        <v>0.22</v>
+        <v>2.31</v>
       </c>
     </row>
     <row r="20">
@@ -16129,19 +16129,19 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>3969</v>
+        <v>5247.9</v>
       </c>
       <c r="M5" t="n">
-        <v>57</v>
+        <v>251.4</v>
       </c>
       <c r="N5" t="n">
         <v>0</v>
       </c>
       <c r="O5" t="n">
-        <v>483</v>
+        <v>534</v>
       </c>
       <c r="P5" t="n">
-        <v>270</v>
+        <v>108</v>
       </c>
       <c r="Q5" t="n">
         <v>25.84</v>
@@ -16182,19 +16182,19 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>2475.3</v>
+        <v>6582.3</v>
       </c>
       <c r="M6" t="n">
-        <v>86.40000000000001</v>
+        <v>753.6</v>
       </c>
       <c r="N6" t="n">
         <v>0</v>
       </c>
       <c r="O6" t="n">
-        <v>390</v>
+        <v>885</v>
       </c>
       <c r="P6" t="n">
-        <v>2497.5</v>
+        <v>1539</v>
       </c>
       <c r="Q6" t="n">
         <v>70.48</v>
@@ -16235,19 +16235,19 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>1566</v>
+        <v>10656</v>
       </c>
       <c r="M7" t="n">
+        <v>2604</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" t="n">
         <v>105</v>
       </c>
-      <c r="N7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O7" t="n">
-        <v>63</v>
-      </c>
       <c r="P7" t="n">
-        <v>3742.5</v>
+        <v>4545</v>
       </c>
       <c r="Q7" t="n">
         <v>25.89</v>
@@ -16288,10 +16288,10 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>1427.1</v>
+        <v>10181.4</v>
       </c>
       <c r="M8" t="n">
-        <v>82.5</v>
+        <v>1881</v>
       </c>
       <c r="N8" t="n">
         <v>0</v>
@@ -16300,7 +16300,7 @@
         <v>0</v>
       </c>
       <c r="P8" t="n">
-        <v>5631.6</v>
+        <v>7615.2</v>
       </c>
       <c r="Q8" t="n">
         <v>27.99</v>
@@ -16341,19 +16341,19 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>1239.3</v>
+        <v>12879</v>
       </c>
       <c r="M9" t="n">
-        <v>105</v>
+        <v>1008</v>
       </c>
       <c r="N9" t="n">
         <v>0</v>
       </c>
       <c r="O9" t="n">
-        <v>0</v>
+        <v>16.5</v>
       </c>
       <c r="P9" t="n">
-        <v>8280</v>
+        <v>14385</v>
       </c>
       <c r="Q9" t="n">
         <v>19.92</v>
@@ -16394,10 +16394,10 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>480.6</v>
+        <v>4165.2</v>
       </c>
       <c r="M10" t="n">
-        <v>102</v>
+        <v>153</v>
       </c>
       <c r="N10" t="n">
         <v>0</v>
@@ -16406,7 +16406,7 @@
         <v>0</v>
       </c>
       <c r="P10" t="n">
-        <v>4411.5</v>
+        <v>10429.5</v>
       </c>
       <c r="Q10" t="n">
         <v>6.25</v>
@@ -16447,7 +16447,7 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>0</v>
+        <v>1050</v>
       </c>
       <c r="M11" t="n">
         <v>0</v>
@@ -16459,7 +16459,7 @@
         <v>0</v>
       </c>
       <c r="P11" t="n">
-        <v>1269</v>
+        <v>4590</v>
       </c>
       <c r="Q11" t="n">
         <v>2.79</v>
@@ -16500,7 +16500,7 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>30</v>
+        <v>390</v>
       </c>
       <c r="M12" t="n">
         <v>0</v>
@@ -16512,7 +16512,7 @@
         <v>0</v>
       </c>
       <c r="P12" t="n">
-        <v>120</v>
+        <v>570</v>
       </c>
       <c r="Q12" t="n">
         <v>1</v>
@@ -16553,7 +16553,7 @@
         <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="M13" t="n">
         <v>0</v>
@@ -16565,7 +16565,7 @@
         <v>0</v>
       </c>
       <c r="P13" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="Q13" t="n">
         <v>0.11</v>
@@ -17421,19 +17421,19 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>714420</v>
+        <v>944622</v>
       </c>
       <c r="M5" t="n">
-        <v>19950</v>
+        <v>87990</v>
       </c>
       <c r="N5" t="n">
         <v>0</v>
       </c>
       <c r="O5" t="n">
-        <v>82110</v>
+        <v>90780</v>
       </c>
       <c r="P5" t="n">
-        <v>17550</v>
+        <v>7020</v>
       </c>
       <c r="Q5" t="n">
         <v>15504.59</v>
@@ -17474,19 +17474,19 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>445554</v>
+        <v>1184814</v>
       </c>
       <c r="M6" t="n">
-        <v>30240</v>
+        <v>263760</v>
       </c>
       <c r="N6" t="n">
         <v>0</v>
       </c>
       <c r="O6" t="n">
-        <v>66300</v>
+        <v>150450</v>
       </c>
       <c r="P6" t="n">
-        <v>162337.5</v>
+        <v>100035</v>
       </c>
       <c r="Q6" t="n">
         <v>42285.24</v>
@@ -17527,19 +17527,19 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>281880</v>
+        <v>1918080</v>
       </c>
       <c r="M7" t="n">
-        <v>36750</v>
+        <v>911400</v>
       </c>
       <c r="N7" t="n">
         <v>0</v>
       </c>
       <c r="O7" t="n">
-        <v>10710</v>
+        <v>17850</v>
       </c>
       <c r="P7" t="n">
-        <v>243262.5</v>
+        <v>295425</v>
       </c>
       <c r="Q7" t="n">
         <v>15534.72</v>
@@ -17580,10 +17580,10 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>256878</v>
+        <v>1832652</v>
       </c>
       <c r="M8" t="n">
-        <v>28875</v>
+        <v>658350</v>
       </c>
       <c r="N8" t="n">
         <v>0</v>
@@ -17592,7 +17592,7 @@
         <v>0</v>
       </c>
       <c r="P8" t="n">
-        <v>366054</v>
+        <v>494988</v>
       </c>
       <c r="Q8" t="n">
         <v>16793.57</v>
@@ -17633,19 +17633,19 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>223074</v>
+        <v>2318220</v>
       </c>
       <c r="M9" t="n">
-        <v>36750</v>
+        <v>352800</v>
       </c>
       <c r="N9" t="n">
         <v>0</v>
       </c>
       <c r="O9" t="n">
-        <v>0</v>
+        <v>2805</v>
       </c>
       <c r="P9" t="n">
-        <v>538200</v>
+        <v>935025</v>
       </c>
       <c r="Q9" t="n">
         <v>11951.02</v>
@@ -17686,10 +17686,10 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>86508</v>
+        <v>749736</v>
       </c>
       <c r="M10" t="n">
-        <v>35700</v>
+        <v>53550</v>
       </c>
       <c r="N10" t="n">
         <v>0</v>
@@ -17698,7 +17698,7 @@
         <v>0</v>
       </c>
       <c r="P10" t="n">
-        <v>286747.5</v>
+        <v>677917.5</v>
       </c>
       <c r="Q10" t="n">
         <v>3749.76</v>
@@ -17739,7 +17739,7 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>0</v>
+        <v>189000</v>
       </c>
       <c r="M11" t="n">
         <v>0</v>
@@ -17751,7 +17751,7 @@
         <v>0</v>
       </c>
       <c r="P11" t="n">
-        <v>82485</v>
+        <v>298350</v>
       </c>
       <c r="Q11" t="n">
         <v>1674</v>
@@ -17792,7 +17792,7 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>5400</v>
+        <v>70200</v>
       </c>
       <c r="M12" t="n">
         <v>0</v>
@@ -17804,7 +17804,7 @@
         <v>0</v>
       </c>
       <c r="P12" t="n">
-        <v>7800</v>
+        <v>37050</v>
       </c>
       <c r="Q12" t="n">
         <v>602.64</v>
@@ -17845,7 +17845,7 @@
         <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>0</v>
+        <v>21600</v>
       </c>
       <c r="M13" t="n">
         <v>0</v>
@@ -17857,7 +17857,7 @@
         <v>0</v>
       </c>
       <c r="P13" t="n">
-        <v>1950</v>
+        <v>5850</v>
       </c>
       <c r="Q13" t="n">
         <v>66.95999999999999</v>
@@ -18660,7 +18660,7 @@
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>300</v>
+        <v>630</v>
       </c>
       <c r="M4" t="n">
         <v>0</v>
@@ -18669,13 +18669,13 @@
         <v>0</v>
       </c>
       <c r="O4" t="n">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="P4" t="n">
-        <v>30</v>
+        <v>240</v>
       </c>
       <c r="Q4" t="n">
-        <v>4.49</v>
+        <v>51.48</v>
       </c>
     </row>
     <row r="5">
@@ -18728,7 +18728,7 @@
         <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.09</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="6">
@@ -20020,7 +20020,7 @@
         <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="6">
@@ -21312,7 +21312,7 @@
         <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>2.59</v>
+        <v>29.7</v>
       </c>
     </row>
     <row r="6">
@@ -22577,7 +22577,7 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>3878280</v>
+        <v>3632040</v>
       </c>
       <c r="I5" t="n">
         <v>64288.14</v>
@@ -22589,22 +22589,22 @@
         <v>176792.4</v>
       </c>
       <c r="L5" t="n">
-        <v>3541482</v>
+        <v>4097142</v>
       </c>
       <c r="M5" t="n">
-        <v>102690</v>
+        <v>248010</v>
       </c>
       <c r="N5" t="n">
-        <v>2397</v>
+        <v>2601</v>
       </c>
       <c r="O5" t="n">
-        <v>87975</v>
+        <v>101235</v>
       </c>
       <c r="P5" t="n">
-        <v>56199</v>
+        <v>42471</v>
       </c>
       <c r="Q5" t="n">
-        <v>502273.66</v>
+        <v>5205013.29</v>
       </c>
     </row>
     <row r="6">
@@ -22630,7 +22630,7 @@
         <v>54594</v>
       </c>
       <c r="H6" t="n">
-        <v>10916640</v>
+        <v>12476160</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
@@ -22642,22 +22642,22 @@
         <v>49235.78</v>
       </c>
       <c r="L6" t="n">
-        <v>4171824</v>
+        <v>5624370</v>
       </c>
       <c r="M6" t="n">
-        <v>174720</v>
+        <v>608160</v>
       </c>
       <c r="N6" t="n">
-        <v>1530</v>
+        <v>3825</v>
       </c>
       <c r="O6" t="n">
-        <v>68850</v>
+        <v>155550</v>
       </c>
       <c r="P6" t="n">
-        <v>367380</v>
+        <v>382005</v>
       </c>
       <c r="Q6" t="n">
-        <v>8306538.66</v>
+        <v>86079856.28</v>
       </c>
     </row>
     <row r="7">
@@ -22683,7 +22683,7 @@
         <v>99630</v>
       </c>
       <c r="H7" t="n">
-        <v>374490</v>
+        <v>1872450</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
@@ -22695,22 +22695,22 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>3836160</v>
+        <v>6648480</v>
       </c>
       <c r="M7" t="n">
-        <v>393225</v>
+        <v>2109450</v>
       </c>
       <c r="N7" t="n">
         <v>0</v>
       </c>
       <c r="O7" t="n">
-        <v>10710</v>
+        <v>23205</v>
       </c>
       <c r="P7" t="n">
-        <v>547462.5</v>
+        <v>730275</v>
       </c>
       <c r="Q7" t="n">
-        <v>6594702.91</v>
+        <v>68340268.08</v>
       </c>
     </row>
     <row r="8">
@@ -22748,10 +22748,10 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>2200716</v>
+        <v>4688982</v>
       </c>
       <c r="M8" t="n">
-        <v>617925</v>
+        <v>1830675</v>
       </c>
       <c r="N8" t="n">
         <v>0</v>
@@ -22760,10 +22760,10 @@
         <v>0</v>
       </c>
       <c r="P8" t="n">
-        <v>551304</v>
+        <v>825474</v>
       </c>
       <c r="Q8" t="n">
-        <v>4834130.33</v>
+        <v>50095624.77</v>
       </c>
     </row>
     <row r="9">
@@ -22789,7 +22789,7 @@
         <v>108783</v>
       </c>
       <c r="H9" t="n">
-        <v>342000</v>
+        <v>1026000</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
@@ -22801,22 +22801,22 @@
         <v>77980.94</v>
       </c>
       <c r="L9" t="n">
-        <v>734832</v>
+        <v>3175524</v>
       </c>
       <c r="M9" t="n">
-        <v>235200</v>
+        <v>1006950</v>
       </c>
       <c r="N9" t="n">
         <v>0</v>
       </c>
       <c r="O9" t="n">
-        <v>0</v>
+        <v>2805</v>
       </c>
       <c r="P9" t="n">
-        <v>757575</v>
+        <v>1302600</v>
       </c>
       <c r="Q9" t="n">
-        <v>2628250.31</v>
+        <v>27236303.6</v>
       </c>
     </row>
     <row r="10">
@@ -22854,10 +22854,10 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>341226</v>
+        <v>1148634</v>
       </c>
       <c r="M10" t="n">
-        <v>62475</v>
+        <v>740775</v>
       </c>
       <c r="N10" t="n">
         <v>0</v>
@@ -22866,10 +22866,10 @@
         <v>0</v>
       </c>
       <c r="P10" t="n">
-        <v>440895</v>
+        <v>853612.5</v>
       </c>
       <c r="Q10" t="n">
-        <v>1352993.76</v>
+        <v>14020943.4</v>
       </c>
     </row>
     <row r="11">
@@ -22907,10 +22907,10 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>264600</v>
+        <v>675000</v>
       </c>
       <c r="M11" t="n">
-        <v>0</v>
+        <v>1587600</v>
       </c>
       <c r="N11" t="n">
         <v>0</v>
@@ -22919,10 +22919,10 @@
         <v>0</v>
       </c>
       <c r="P11" t="n">
-        <v>301860</v>
+        <v>814320</v>
       </c>
       <c r="Q11" t="n">
-        <v>812023.92</v>
+        <v>8414925.300000001</v>
       </c>
     </row>
     <row r="12">
@@ -22960,10 +22960,10 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>64800</v>
+        <v>367200</v>
       </c>
       <c r="M12" t="n">
-        <v>0</v>
+        <v>309225</v>
       </c>
       <c r="N12" t="n">
         <v>0</v>
@@ -22972,10 +22972,10 @@
         <v>0</v>
       </c>
       <c r="P12" t="n">
-        <v>42900</v>
+        <v>136500</v>
       </c>
       <c r="Q12" t="n">
-        <v>620250.48</v>
+        <v>6427595.7</v>
       </c>
     </row>
     <row r="13">
@@ -23001,7 +23001,7 @@
         <v>8100</v>
       </c>
       <c r="H13" t="n">
-        <v>171000</v>
+        <v>513000</v>
       </c>
       <c r="I13" t="n">
         <v>0</v>
@@ -23013,10 +23013,10 @@
         <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>43200</v>
+        <v>118800</v>
       </c>
       <c r="M13" t="n">
-        <v>0</v>
+        <v>31500</v>
       </c>
       <c r="N13" t="n">
         <v>0</v>
@@ -23025,10 +23025,10 @@
         <v>0</v>
       </c>
       <c r="P13" t="n">
-        <v>1950</v>
+        <v>5850</v>
       </c>
       <c r="Q13" t="n">
-        <v>626544.72</v>
+        <v>6492822.3</v>
       </c>
     </row>
     <row r="14">
@@ -23066,10 +23066,10 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>97200</v>
+        <v>253800</v>
       </c>
       <c r="M14" t="n">
-        <v>0</v>
+        <v>52500</v>
       </c>
       <c r="N14" t="n">
         <v>0</v>
@@ -23081,7 +23081,7 @@
         <v>0</v>
       </c>
       <c r="Q14" t="n">
-        <v>652926.96</v>
+        <v>6766218.9</v>
       </c>
     </row>
     <row r="15">
@@ -23119,10 +23119,10 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>0</v>
+        <v>172800</v>
       </c>
       <c r="M15" t="n">
-        <v>0</v>
+        <v>84000</v>
       </c>
       <c r="N15" t="n">
         <v>0</v>
@@ -23134,7 +23134,7 @@
         <v>0</v>
       </c>
       <c r="Q15" t="n">
-        <v>279290.16</v>
+        <v>2894256.9</v>
       </c>
     </row>
     <row r="16">
@@ -23172,7 +23172,7 @@
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>0</v>
+        <v>64800</v>
       </c>
       <c r="M16" t="n">
         <v>0</v>
@@ -23187,7 +23187,7 @@
         <v>0</v>
       </c>
       <c r="Q16" t="n">
-        <v>104524.56</v>
+        <v>1083177.9</v>
       </c>
     </row>
     <row r="17">
@@ -23225,7 +23225,7 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>0</v>
+        <v>16200</v>
       </c>
       <c r="M17" t="n">
         <v>0</v>
@@ -23240,7 +23240,7 @@
         <v>0</v>
       </c>
       <c r="Q17" t="n">
-        <v>22096.8</v>
+        <v>228987</v>
       </c>
     </row>
     <row r="18">
@@ -23278,7 +23278,7 @@
         <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>0</v>
+        <v>27000</v>
       </c>
       <c r="M18" t="n">
         <v>0</v>
@@ -23293,7 +23293,7 @@
         <v>0</v>
       </c>
       <c r="Q18" t="n">
-        <v>2209.68</v>
+        <v>22898.7</v>
       </c>
     </row>
     <row r="19">
@@ -23346,7 +23346,7 @@
         <v>0</v>
       </c>
       <c r="Q19" t="n">
-        <v>133.92</v>
+        <v>1387.8</v>
       </c>
     </row>
     <row r="20">
@@ -23828,22 +23828,22 @@
         <v>2</v>
       </c>
       <c r="L4" t="n">
-        <v>22350</v>
+        <v>25440</v>
       </c>
       <c r="M4" t="n">
-        <v>9420</v>
+        <v>15240</v>
       </c>
       <c r="N4" t="n">
-        <v>2550</v>
+        <v>3480</v>
       </c>
       <c r="O4" t="n">
-        <v>3390</v>
+        <v>3210</v>
       </c>
       <c r="P4" t="n">
-        <v>2370</v>
+        <v>4230</v>
       </c>
       <c r="Q4" t="n">
-        <v>1787.07</v>
+        <v>17520.3</v>
       </c>
     </row>
     <row r="5">
@@ -23881,22 +23881,22 @@
         <v>4</v>
       </c>
       <c r="L5" t="n">
-        <v>26910</v>
+        <v>31260</v>
       </c>
       <c r="M5" t="n">
-        <v>1800</v>
+        <v>4140</v>
       </c>
       <c r="N5" t="n">
-        <v>1410</v>
+        <v>1500</v>
       </c>
       <c r="O5" t="n">
-        <v>690</v>
+        <v>1230</v>
       </c>
       <c r="P5" t="n">
-        <v>4140</v>
+        <v>5250</v>
       </c>
       <c r="Q5" t="n">
-        <v>3276.53</v>
+        <v>32122.8</v>
       </c>
     </row>
     <row r="6">
@@ -23934,22 +23934,22 @@
         <v>1</v>
       </c>
       <c r="L6" t="n">
-        <v>15840</v>
+        <v>19230</v>
       </c>
       <c r="M6" t="n">
-        <v>0</v>
+        <v>270</v>
       </c>
       <c r="N6" t="n">
-        <v>180</v>
+        <v>450</v>
       </c>
       <c r="O6" t="n">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="P6" t="n">
         <v>3630</v>
       </c>
       <c r="Q6" t="n">
-        <v>3517.13</v>
+        <v>34481.7</v>
       </c>
     </row>
     <row r="7">
@@ -23987,7 +23987,7 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>7020</v>
+        <v>8370</v>
       </c>
       <c r="M7" t="n">
         <v>0</v>
@@ -23996,13 +23996,13 @@
         <v>0</v>
       </c>
       <c r="O7" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="P7" t="n">
-        <v>4440</v>
+        <v>4920</v>
       </c>
       <c r="Q7" t="n">
-        <v>1890.8</v>
+        <v>18537.3</v>
       </c>
     </row>
     <row r="8">
@@ -24040,7 +24040,7 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>2160</v>
+        <v>2760</v>
       </c>
       <c r="M8" t="n">
         <v>0</v>
@@ -24052,10 +24052,10 @@
         <v>0</v>
       </c>
       <c r="P8" t="n">
-        <v>1320</v>
+        <v>3150</v>
       </c>
       <c r="Q8" t="n">
-        <v>853.5599999999999</v>
+        <v>8368.200000000001</v>
       </c>
     </row>
     <row r="9">
@@ -24093,7 +24093,7 @@
         <v>1</v>
       </c>
       <c r="L9" t="n">
-        <v>720</v>
+        <v>960</v>
       </c>
       <c r="M9" t="n">
         <v>0</v>
@@ -24108,7 +24108,7 @@
         <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>304.59</v>
+        <v>2986.2</v>
       </c>
     </row>
     <row r="10">
@@ -24146,7 +24146,7 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>270</v>
+        <v>300</v>
       </c>
       <c r="M10" t="n">
         <v>0</v>
@@ -24161,7 +24161,7 @@
         <v>0</v>
       </c>
       <c r="Q10" t="n">
-        <v>108.6</v>
+        <v>1064.7</v>
       </c>
     </row>
     <row r="11">
@@ -24199,7 +24199,7 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>30</v>
+        <v>180</v>
       </c>
       <c r="M11" t="n">
         <v>0</v>
@@ -24214,7 +24214,7 @@
         <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>53.06</v>
+        <v>520.2</v>
       </c>
     </row>
     <row r="12">
@@ -24252,7 +24252,7 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="M12" t="n">
         <v>0</v>
@@ -24267,7 +24267,7 @@
         <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>35.8</v>
+        <v>351</v>
       </c>
     </row>
     <row r="13">
@@ -24320,7 +24320,7 @@
         <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>22.22</v>
+        <v>217.8</v>
       </c>
     </row>
     <row r="14">
@@ -24373,7 +24373,7 @@
         <v>0</v>
       </c>
       <c r="Q14" t="n">
-        <v>23.5</v>
+        <v>230.4</v>
       </c>
     </row>
     <row r="15">
@@ -25173,22 +25173,22 @@
         <v>1.32</v>
       </c>
       <c r="L5" t="n">
-        <v>5651.1</v>
+        <v>6564.6</v>
       </c>
       <c r="M5" t="n">
-        <v>36</v>
+        <v>82.8</v>
       </c>
       <c r="N5" t="n">
-        <v>14.1</v>
+        <v>15</v>
       </c>
       <c r="O5" t="n">
-        <v>34.5</v>
+        <v>61.5</v>
       </c>
       <c r="P5" t="n">
-        <v>82.8</v>
+        <v>105</v>
       </c>
       <c r="Q5" t="n">
-        <v>163.83</v>
+        <v>1606.14</v>
       </c>
     </row>
     <row r="6">
@@ -25226,22 +25226,22 @@
         <v>0.51</v>
       </c>
       <c r="L6" t="n">
-        <v>5860.8</v>
+        <v>7115.1</v>
       </c>
       <c r="M6" t="n">
-        <v>0</v>
+        <v>21.6</v>
       </c>
       <c r="N6" t="n">
-        <v>9</v>
+        <v>22.5</v>
       </c>
       <c r="O6" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="P6" t="n">
         <v>544.5</v>
       </c>
       <c r="Q6" t="n">
-        <v>2637.85</v>
+        <v>25861.28</v>
       </c>
     </row>
     <row r="7">
@@ -25279,7 +25279,7 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>4212</v>
+        <v>5022</v>
       </c>
       <c r="M7" t="n">
         <v>0</v>
@@ -25288,13 +25288,13 @@
         <v>0</v>
       </c>
       <c r="O7" t="n">
-        <v>0</v>
+        <v>31.5</v>
       </c>
       <c r="P7" t="n">
-        <v>1110</v>
+        <v>1230</v>
       </c>
       <c r="Q7" t="n">
-        <v>1512.64</v>
+        <v>14829.84</v>
       </c>
     </row>
     <row r="8">
@@ -25332,7 +25332,7 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>1533.6</v>
+        <v>1959.6</v>
       </c>
       <c r="M8" t="n">
         <v>0</v>
@@ -25344,10 +25344,10 @@
         <v>0</v>
       </c>
       <c r="P8" t="n">
-        <v>501.6</v>
+        <v>1197</v>
       </c>
       <c r="Q8" t="n">
-        <v>810.88</v>
+        <v>7949.79</v>
       </c>
     </row>
     <row r="9">
@@ -25385,7 +25385,7 @@
         <v>0.8</v>
       </c>
       <c r="L9" t="n">
-        <v>583.2</v>
+        <v>777.6</v>
       </c>
       <c r="M9" t="n">
         <v>0</v>
@@ -25400,7 +25400,7 @@
         <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>295.45</v>
+        <v>2896.61</v>
       </c>
     </row>
     <row r="10">
@@ -25438,7 +25438,7 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>240.3</v>
+        <v>267</v>
       </c>
       <c r="M10" t="n">
         <v>0</v>
@@ -25453,7 +25453,7 @@
         <v>0</v>
       </c>
       <c r="Q10" t="n">
-        <v>108.6</v>
+        <v>1064.7</v>
       </c>
     </row>
     <row r="11">
@@ -25491,7 +25491,7 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>30</v>
+        <v>180</v>
       </c>
       <c r="M11" t="n">
         <v>0</v>
@@ -25506,7 +25506,7 @@
         <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>53.06</v>
+        <v>520.2</v>
       </c>
     </row>
     <row r="12">
@@ -25544,7 +25544,7 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="M12" t="n">
         <v>0</v>
@@ -25559,7 +25559,7 @@
         <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>35.8</v>
+        <v>351</v>
       </c>
     </row>
     <row r="13">
@@ -25612,7 +25612,7 @@
         <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>22.22</v>
+        <v>217.8</v>
       </c>
     </row>
     <row r="14">
@@ -25665,7 +25665,7 @@
         <v>0</v>
       </c>
       <c r="Q14" t="n">
-        <v>23.5</v>
+        <v>230.4</v>
       </c>
     </row>
     <row r="15">
@@ -26465,22 +26465,22 @@
         <v>64288.14</v>
       </c>
       <c r="L5" t="n">
-        <v>1017198</v>
+        <v>1181628</v>
       </c>
       <c r="M5" t="n">
-        <v>12600</v>
+        <v>28980</v>
       </c>
       <c r="N5" t="n">
-        <v>2397</v>
+        <v>2550</v>
       </c>
       <c r="O5" t="n">
-        <v>5865</v>
+        <v>10455</v>
       </c>
       <c r="P5" t="n">
-        <v>5382</v>
+        <v>6825</v>
       </c>
       <c r="Q5" t="n">
-        <v>98295.77</v>
+        <v>963684</v>
       </c>
     </row>
     <row r="6">
@@ -26518,22 +26518,22 @@
         <v>24617.89</v>
       </c>
       <c r="L6" t="n">
-        <v>1054944</v>
+        <v>1280718</v>
       </c>
       <c r="M6" t="n">
-        <v>0</v>
+        <v>7560</v>
       </c>
       <c r="N6" t="n">
-        <v>1530</v>
+        <v>3825</v>
       </c>
       <c r="O6" t="n">
-        <v>2550</v>
+        <v>5100</v>
       </c>
       <c r="P6" t="n">
         <v>35392.5</v>
       </c>
       <c r="Q6" t="n">
-        <v>1582710.03</v>
+        <v>15516765</v>
       </c>
     </row>
     <row r="7">
@@ -26571,7 +26571,7 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>758160</v>
+        <v>903960</v>
       </c>
       <c r="M7" t="n">
         <v>0</v>
@@ -26580,13 +26580,13 @@
         <v>0</v>
       </c>
       <c r="O7" t="n">
-        <v>0</v>
+        <v>5355</v>
       </c>
       <c r="P7" t="n">
-        <v>72150</v>
+        <v>79950</v>
       </c>
       <c r="Q7" t="n">
-        <v>907586.21</v>
+        <v>8897904</v>
       </c>
     </row>
     <row r="8">
@@ -26624,7 +26624,7 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>276048</v>
+        <v>352728</v>
       </c>
       <c r="M8" t="n">
         <v>0</v>
@@ -26636,10 +26636,10 @@
         <v>0</v>
       </c>
       <c r="P8" t="n">
-        <v>32604</v>
+        <v>77805</v>
       </c>
       <c r="Q8" t="n">
-        <v>486527.15</v>
+        <v>4769874</v>
       </c>
     </row>
     <row r="9">
@@ -26677,7 +26677,7 @@
         <v>38990.47</v>
       </c>
       <c r="L9" t="n">
-        <v>104976</v>
+        <v>139968</v>
       </c>
       <c r="M9" t="n">
         <v>0</v>
@@ -26692,7 +26692,7 @@
         <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>177272.78</v>
+        <v>1737968.4</v>
       </c>
     </row>
     <row r="10">
@@ -26730,7 +26730,7 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>43254</v>
+        <v>48060</v>
       </c>
       <c r="M10" t="n">
         <v>0</v>
@@ -26745,7 +26745,7 @@
         <v>0</v>
       </c>
       <c r="Q10" t="n">
-        <v>65159.64</v>
+        <v>638820</v>
       </c>
     </row>
     <row r="11">
@@ -26783,7 +26783,7 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>5400</v>
+        <v>32400</v>
       </c>
       <c r="M11" t="n">
         <v>0</v>
@@ -26798,7 +26798,7 @@
         <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>31836.24</v>
+        <v>312120</v>
       </c>
     </row>
     <row r="12">
@@ -26836,7 +26836,7 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>0</v>
+        <v>5400</v>
       </c>
       <c r="M12" t="n">
         <v>0</v>
@@ -26851,7 +26851,7 @@
         <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>21481.2</v>
+        <v>210600</v>
       </c>
     </row>
     <row r="13">
@@ -26904,7 +26904,7 @@
         <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>13329.36</v>
+        <v>130680</v>
       </c>
     </row>
     <row r="14">
@@ -26957,7 +26957,7 @@
         <v>0</v>
       </c>
       <c r="Q14" t="n">
-        <v>14100.48</v>
+        <v>138240</v>
       </c>
     </row>
     <row r="15">
@@ -27692,7 +27692,7 @@
         <v>540</v>
       </c>
       <c r="H4" t="n">
-        <v>210</v>
+        <v>300</v>
       </c>
       <c r="I4" t="n">
         <v>0</v>
@@ -27704,7 +27704,7 @@
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>510</v>
+        <v>1440</v>
       </c>
       <c r="M4" t="n">
         <v>0</v>
@@ -27713,13 +27713,13 @@
         <v>0</v>
       </c>
       <c r="O4" t="n">
-        <v>360</v>
+        <v>720</v>
       </c>
       <c r="P4" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="Q4" t="n">
-        <v>15.71</v>
+        <v>218.79</v>
       </c>
     </row>
     <row r="5">
@@ -27745,7 +27745,7 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -27757,7 +27757,7 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="M5" t="n">
         <v>0</v>
@@ -29037,7 +29037,7 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>10.8</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -29049,7 +29049,7 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>18.9</v>
       </c>
       <c r="M5" t="n">
         <v>0</v>
@@ -30329,7 +30329,7 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>61560</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -30341,7 +30341,7 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>3402</v>
       </c>
       <c r="M5" t="n">
         <v>0</v>

</xml_diff>